<commit_message>
Release v1.2.2 inference-presentation update
</commit_message>
<xml_diff>
--- a/tables/Table_2_signature_summary.xlsx
+++ b/tables/Table_2_signature_summary.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra0eccc935f584daf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="Rc3cadeec5c124481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc3a6005c9e964c09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" r:id="Rec6c57ec63be4ec7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -59,8 +59,26 @@
       <x:sz val="8"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF244158"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF244158"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -82,16 +100,50 @@
         <x:fgColor rgb="FFEAF2F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE6F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F6B8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA6B4BF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFA6B4BF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFA6B4BF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6B4BF"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="63">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -147,6 +199,103 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -350,70 +499,82 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="88" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="92" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="3" t="str">
-        <x:v>Table 2 source, analysis release v1.2.1</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="str">
-        <x:v>Submission-matched reviewer-facing table</x:v>
+    <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A1" s="37" t="str">
+        <x:v>Table 2 source, release v1.2.2</x:v>
+      </x:c>
+      <x:c r="B1" s="37" t="str">
+        <x:v>Manuscript-facing summary table</x:v>
       </x:c>
       <x:c r="C1" s="3"/>
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
       <x:c r="F1" s="3"/>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
+    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A2" s="35" t="str">
         <x:v>Version boundary</x:v>
       </x:c>
-      <x:c r="B2" t="str">
-        <x:v>Stage 3 score meta-analysis values are unchanged. Stage 4 contribution summaries use the exact signature-specific primary-independent cohort sets.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="6" t="str">
+      <x:c r="B2" s="7" t="str">
+        <x:v>The v1.2.1 numerical workflow, cohorts, point estimates, standard Hartung–Knapp results, prediction intervals, and gene-contribution metrics are unchanged. Version 1.2.2 adds modified Hartung–Knapp intervals and Holm-adjusted P values to the main table and removes the threshold-dependent pattern label.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="35" t="str">
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
-        <x:v>Submission-matched v1.2.1 release</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="6" t="str">
+        <x:v>v1.2.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="35" t="str">
+        <x:v>DOI</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>10.5281/zenodo.21506111</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="35" t="str">
         <x:v>Manuscript</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="B5" s="8" t="str">
         <x:v>Scientific_Reports_Manuscript.docx</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="6" t="str">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="35" t="str">
         <x:v>QC</x:v>
       </x:c>
-      <x:c r="B5" s="8" t="str">
-        <x:v>Values agree with the corrected machine-readable source</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="9" t="str">
+      <x:c r="B6" s="7" t="str">
+        <x:v>Values agree with Supplementary Data Table S25 and the corrected machine-readable sources.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="7"/>
+      <x:c r="B7" s="7"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="38" t="str">
         <x:v>Workbook map</x:v>
       </x:c>
-      <x:c r="B8" s="9"/>
+      <x:c r="B8" s="38"/>
       <x:c r="C8" s="9"/>
       <x:c r="D8" s="9"/>
       <x:c r="E8" s="9"/>
       <x:c r="F8" s="9"/>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="11" t="str">
-        <x:v>v1.2.0 scientific correction retained in v1.2.1</x:v>
+    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A9" s="39" t="str">
+        <x:v>Scientific continuity</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>SIG002, SIG003, and SIG004 contribution metrics use four T48 cohorts and 118 patients. SIG004 is now consistent multigene drift; SIG003 changes in one threshold scenario.</x:v>
+        <x:v>SIG002, SIG003, and SIG004 contribution metrics retain the exact signature-specific primary-independent T48 sets (four study families; 118 patients). Continuous dominance and cancellation metrics are presented without the threshold-dependent pattern label.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -429,17 +590,18 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="8" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="26" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -485,318 +647,345 @@
       <x:c r="J3" s="7"/>
       <x:c r="K3" s="7"/>
     </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="27" t="str">
+    <x:row r="4" ht="44" hidden="0" customHeight="1">
+      <x:c r="A4" s="56" t="str">
         <x:v>Signature</x:v>
       </x:c>
-      <x:c r="B4" s="27" t="str">
+      <x:c r="B4" s="50" t="str">
         <x:v>T24 k</x:v>
       </x:c>
-      <x:c r="C4" s="27" t="str">
-        <x:v>T24 delta Z (95% CI)</x:v>
-      </x:c>
-      <x:c r="D4" s="27" t="str">
+      <x:c r="C4" s="50" t="str">
+        <x:v>T24 delta Z, standard HK (95% CI)</x:v>
+      </x:c>
+      <x:c r="D4" s="50" t="str">
+        <x:v>T24 modified HK (95% CI; Holm P)</x:v>
+      </x:c>
+      <x:c r="E4" s="50" t="str">
         <x:v>T48 k</x:v>
       </x:c>
-      <x:c r="E4" s="27" t="str">
-        <x:v>T48 delta Z (95% CI)</x:v>
-      </x:c>
-      <x:c r="F4" s="27" t="str">
+      <x:c r="F4" s="50" t="str">
+        <x:v>T48 delta Z, standard HK (95% CI)</x:v>
+      </x:c>
+      <x:c r="G4" s="50" t="str">
+        <x:v>T48 modified HK (95% CI; Holm P)</x:v>
+      </x:c>
+      <x:c r="H4" s="50" t="str">
         <x:v>T48 95% PI</x:v>
       </x:c>
-      <x:c r="G4" s="27" t="str">
+      <x:c r="I4" s="50" t="str">
         <x:v>T48 I², %</x:v>
       </x:c>
-      <x:c r="H4" s="27" t="str">
-        <x:v>T48 pattern</x:v>
-      </x:c>
-      <x:c r="I4" s="27" t="str">
+      <x:c r="J4" s="50" t="str">
         <x:v>T48 leading gene</x:v>
       </x:c>
-      <x:c r="J4" s="27" t="str">
+      <x:c r="K4" s="50" t="str">
         <x:v>T48 dominance</x:v>
       </x:c>
-      <x:c r="K4" s="27" t="str">
+      <x:c r="L4" s="51" t="str">
         <x:v>T48 cancellation</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="24" t="str">
+      <x:c r="A5" s="57" t="str">
         <x:v>SIG001</x:v>
       </x:c>
-      <x:c r="B5" s="24" t="str">
+      <x:c r="B5" s="59" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C5" s="24" t="str">
+      <x:c r="C5" s="59" t="str">
         <x:v>-0.379 (-0.432 to -0.325)</x:v>
       </x:c>
-      <x:c r="D5" s="24" t="str">
+      <x:c r="D5" s="59" t="str">
+        <x:v>-0.560 to -0.197; P=0.042</x:v>
+      </x:c>
+      <x:c r="E5" s="59" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E5" s="24" t="str">
+      <x:c r="F5" s="59" t="str">
         <x:v>-0.855 (-1.351 to -0.359)</x:v>
       </x:c>
-      <x:c r="F5" s="24" t="str">
+      <x:c r="G5" s="59" t="str">
+        <x:v>-1.368 to -0.342; P=0.049</x:v>
+      </x:c>
+      <x:c r="H5" s="59" t="str">
         <x:v>-2.176 to 0.466</x:v>
       </x:c>
-      <x:c r="G5" s="24" t="str">
+      <x:c r="I5" s="59" t="str">
         <x:v>87.4</x:v>
       </x:c>
-      <x:c r="H5" s="24" t="str">
-        <x:v>Cohort-dependent</x:v>
-      </x:c>
-      <x:c r="I5" s="24" t="str">
+      <x:c r="J5" s="59" t="str">
         <x:v>CEACAM1</x:v>
       </x:c>
-      <x:c r="J5" s="24" t="str">
+      <x:c r="K5" s="59" t="str">
         <x:v>0.291</x:v>
       </x:c>
-      <x:c r="K5" s="24" t="str">
+      <x:c r="L5" s="60" t="str">
         <x:v>0.295</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="24" t="str">
+      <x:c r="A6" s="58" t="str">
         <x:v>SIG002</x:v>
       </x:c>
-      <x:c r="B6" s="24" t="str">
+      <x:c r="B6" s="61" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C6" s="24" t="str">
+      <x:c r="C6" s="61" t="str">
         <x:v>-0.071 (-0.181 to 0.039)</x:v>
       </x:c>
-      <x:c r="D6" s="24" t="str">
+      <x:c r="D6" s="61" t="str">
+        <x:v>-0.299 to 0.157; P=0.626</x:v>
+      </x:c>
+      <x:c r="E6" s="61" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E6" s="24" t="str">
+      <x:c r="F6" s="61" t="str">
         <x:v>-0.689 (-0.906 to -0.472)</x:v>
       </x:c>
-      <x:c r="F6" s="24" t="str">
+      <x:c r="G6" s="61" t="str">
+        <x:v>-0.980 to -0.397; P=0.034</x:v>
+      </x:c>
+      <x:c r="H6" s="61" t="str">
         <x:v>-0.982 to -0.395</x:v>
       </x:c>
-      <x:c r="G6" s="24" t="str">
+      <x:c r="I6" s="61" t="str">
         <x:v>0.0</x:v>
       </x:c>
-      <x:c r="H6" s="24" t="str">
-        <x:v>Multigene drift†</x:v>
-      </x:c>
-      <x:c r="I6" s="24" t="str">
+      <x:c r="J6" s="61" t="str">
         <x:v>PLAC8</x:v>
       </x:c>
-      <x:c r="J6" s="24" t="str">
+      <x:c r="K6" s="61" t="str">
         <x:v>0.510</x:v>
       </x:c>
-      <x:c r="K6" s="24" t="str">
+      <x:c r="L6" s="62" t="str">
         <x:v>0.490</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="24" t="str">
+      <x:c r="A7" s="57" t="str">
         <x:v>SIG003</x:v>
       </x:c>
-      <x:c r="B7" s="24" t="str">
+      <x:c r="B7" s="59" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C7" s="24" t="str">
+      <x:c r="C7" s="59" t="str">
         <x:v>-0.173 (-0.269 to -0.077)</x:v>
       </x:c>
-      <x:c r="D7" s="24" t="str">
+      <x:c r="D7" s="59" t="str">
+        <x:v>-0.505 to 0.159; P=0.462†</x:v>
+      </x:c>
+      <x:c r="E7" s="59" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E7" s="24" t="str">
+      <x:c r="F7" s="59" t="str">
         <x:v>-0.899 (-1.224 to -0.574)</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="str">
+      <x:c r="G7" s="59" t="str">
+        <x:v>-1.242 to -0.556; P=0.029</x:v>
+      </x:c>
+      <x:c r="H7" s="59" t="str">
         <x:v>-1.354 to -0.444</x:v>
       </x:c>
-      <x:c r="G7" s="24" t="str">
+      <x:c r="I7" s="59" t="str">
         <x:v>0.0</x:v>
       </x:c>
-      <x:c r="H7" s="24" t="str">
-        <x:v>Single-gene dominant‡</x:v>
-      </x:c>
-      <x:c r="I7" s="24" t="str">
+      <x:c r="J7" s="59" t="str">
         <x:v>PLAC8</x:v>
       </x:c>
-      <x:c r="J7" s="24" t="str">
+      <x:c r="K7" s="59" t="str">
         <x:v>0.679</x:v>
       </x:c>
-      <x:c r="K7" s="24" t="str">
+      <x:c r="L7" s="60" t="str">
         <x:v>0.000</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="24" t="str">
+      <x:c r="A8" s="58" t="str">
         <x:v>SIG004</x:v>
       </x:c>
-      <x:c r="B8" s="24" t="str">
+      <x:c r="B8" s="61" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C8" s="24" t="str">
+      <x:c r="C8" s="61" t="str">
         <x:v>0.027 (-0.378 to 0.431)</x:v>
       </x:c>
-      <x:c r="D8" s="24" t="str">
+      <x:c r="D8" s="61" t="str">
+        <x:v>-0.390 to 0.444; P=0.807</x:v>
+      </x:c>
+      <x:c r="E8" s="61" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E8" s="24" t="str">
+      <x:c r="F8" s="61" t="str">
         <x:v>0.697 (0.332 to 1.062)</x:v>
       </x:c>
-      <x:c r="F8" s="24" t="str">
+      <x:c r="G8" s="61" t="str">
+        <x:v>0.281 to 1.114; P=0.052†</x:v>
+      </x:c>
+      <x:c r="H8" s="61" t="str">
         <x:v>-0.150 to 1.544</x:v>
       </x:c>
-      <x:c r="G8" s="24" t="str">
+      <x:c r="I8" s="61" t="str">
         <x:v>31.2</x:v>
       </x:c>
-      <x:c r="H8" s="24" t="str">
-        <x:v>Multigene drift†</x:v>
-      </x:c>
-      <x:c r="I8" s="24" t="str">
+      <x:c r="J8" s="61" t="str">
         <x:v>NLRP1</x:v>
       </x:c>
-      <x:c r="J8" s="24" t="str">
+      <x:c r="K8" s="61" t="str">
         <x:v>0.589</x:v>
       </x:c>
-      <x:c r="K8" s="24" t="str">
+      <x:c r="L8" s="62" t="str">
         <x:v>0.345</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="24" t="str">
+      <x:c r="A9" s="57" t="str">
         <x:v>SIG022</x:v>
       </x:c>
-      <x:c r="B9" s="24" t="str">
+      <x:c r="B9" s="59" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C9" s="24" t="str">
+      <x:c r="C9" s="59" t="str">
         <x:v>-0.057 (-0.315 to 0.202)</x:v>
       </x:c>
-      <x:c r="D9" s="24" t="str">
+      <x:c r="D9" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E9" s="59" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E9" s="24" t="str">
+      <x:c r="F9" s="59" t="str">
         <x:v>0.139 (-0.191 to 0.469)</x:v>
       </x:c>
-      <x:c r="F9" s="24" t="str">
+      <x:c r="G9" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H9" s="59" t="str">
         <x:v>-0.720 to 0.998</x:v>
       </x:c>
-      <x:c r="G9" s="24" t="str">
+      <x:c r="I9" s="59" t="str">
         <x:v>82.2</x:v>
       </x:c>
-      <x:c r="H9" s="24" t="str">
-        <x:v>Cohort-dependent</x:v>
-      </x:c>
-      <x:c r="I9" s="24" t="str">
+      <x:c r="J9" s="59" t="str">
         <x:v>HK3</x:v>
       </x:c>
-      <x:c r="J9" s="24" t="str">
+      <x:c r="K9" s="59" t="str">
         <x:v>0.389</x:v>
       </x:c>
-      <x:c r="K9" s="24" t="str">
+      <x:c r="L9" s="60" t="str">
         <x:v>0.507</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="24" t="str">
+      <x:c r="A10" s="58" t="str">
         <x:v>SIG023</x:v>
       </x:c>
-      <x:c r="B10" s="24" t="str">
+      <x:c r="B10" s="61" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C10" s="24" t="str">
+      <x:c r="C10" s="61" t="str">
         <x:v>0.047 (-0.523 to 0.617)</x:v>
       </x:c>
-      <x:c r="D10" s="24" t="str">
+      <x:c r="D10" s="61" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E10" s="24" t="str">
+      <x:c r="F10" s="61" t="str">
         <x:v>-0.053 (-0.274 to 0.169)</x:v>
       </x:c>
-      <x:c r="F10" s="24" t="str">
+      <x:c r="G10" s="61" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H10" s="61" t="str">
         <x:v>-0.520 to 0.414</x:v>
       </x:c>
-      <x:c r="G10" s="24" t="str">
+      <x:c r="I10" s="61" t="str">
         <x:v>44.1</x:v>
       </x:c>
-      <x:c r="H10" s="24" t="str">
-        <x:v>Single-gene dominant</x:v>
-      </x:c>
-      <x:c r="I10" s="24" t="str">
+      <x:c r="J10" s="61" t="str">
         <x:v>FAM89A</x:v>
       </x:c>
-      <x:c r="J10" s="24" t="str">
+      <x:c r="K10" s="61" t="str">
         <x:v>0.735</x:v>
       </x:c>
-      <x:c r="K10" s="24" t="str">
+      <x:c r="L10" s="62" t="str">
         <x:v>0.000</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="24" t="str">
+      <x:c r="A11" s="57" t="str">
         <x:v>SIG033</x:v>
       </x:c>
-      <x:c r="B11" s="24" t="str">
+      <x:c r="B11" s="59" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C11" s="24" t="str">
+      <x:c r="C11" s="59" t="str">
         <x:v>-0.162 (-0.358 to 0.033)</x:v>
       </x:c>
-      <x:c r="D11" s="24" t="str">
+      <x:c r="D11" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E11" s="59" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E11" s="24" t="str">
+      <x:c r="F11" s="59" t="str">
         <x:v>-0.120 (-0.365 to 0.125)</x:v>
       </x:c>
-      <x:c r="F11" s="24" t="str">
+      <x:c r="G11" s="59" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H11" s="59" t="str">
         <x:v>-0.468 to 0.228</x:v>
       </x:c>
-      <x:c r="G11" s="24" t="str">
+      <x:c r="I11" s="59" t="str">
         <x:v>18.5</x:v>
       </x:c>
-      <x:c r="H11" s="24" t="str">
-        <x:v>Cohort-dependent</x:v>
-      </x:c>
-      <x:c r="I11" s="24" t="str">
+      <x:c r="J11" s="59" t="str">
         <x:v>LTB</x:v>
       </x:c>
-      <x:c r="J11" s="24" t="str">
+      <x:c r="K11" s="59" t="str">
         <x:v>0.339</x:v>
       </x:c>
-      <x:c r="K11" s="24" t="str">
+      <x:c r="L11" s="60" t="str">
         <x:v>0.610</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="24" t="str">
+      <x:c r="A12" s="58" t="str">
         <x:v>SIG034</x:v>
       </x:c>
-      <x:c r="B12" s="24" t="str">
+      <x:c r="B12" s="61" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C12" s="24" t="str">
+      <x:c r="C12" s="61" t="str">
         <x:v>0.030 (-0.128 to 0.188)</x:v>
       </x:c>
-      <x:c r="D12" s="24" t="str">
+      <x:c r="D12" s="61" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E12" s="61" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E12" s="24" t="str">
+      <x:c r="F12" s="61" t="str">
         <x:v>-0.070 (-0.283 to 0.142)</x:v>
       </x:c>
-      <x:c r="F12" s="24" t="str">
+      <x:c r="G12" s="61" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="H12" s="61" t="str">
         <x:v>-0.451 to 0.310</x:v>
       </x:c>
-      <x:c r="G12" s="24" t="str">
+      <x:c r="I12" s="61" t="str">
         <x:v>18.9</x:v>
       </x:c>
-      <x:c r="H12" s="24" t="str">
-        <x:v>Cohort-dependent</x:v>
-      </x:c>
-      <x:c r="I12" s="24" t="str">
+      <x:c r="J12" s="61" t="str">
         <x:v>DEFA4</x:v>
       </x:c>
-      <x:c r="J12" s="24" t="str">
+      <x:c r="K12" s="61" t="str">
         <x:v>0.098</x:v>
       </x:c>
-      <x:c r="K12" s="24" t="str">
+      <x:c r="L12" s="62" t="str">
         <x:v>0.773</x:v>
       </x:c>
     </x:row>

</xml_diff>